<commit_message>
Updated documents to support I-17_CORS_Origin_Implementation_Steps implementation.
</commit_message>
<xml_diff>
--- a/planing/implementation-plan/azure-policy-assist-prioritized-implementation-log-v12.xlsx
+++ b/planing/implementation-plan/azure-policy-assist-prioritized-implementation-log-v12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steven\GitHub-Repositories\Repositories\azure-policy-assistant-rag-solution-docs\planing\implementation-plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAC4773A-53AB-4C7A-9955-B59E3DA52FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{745A0F1F-4CB1-4E77-BFF2-63B2EC617C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="14235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Policy Implementation Backlog" sheetId="1" r:id="rId1"/>
@@ -1128,7 +1128,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="34" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1338,6 +1338,20 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="8"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1654,7 +1668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1735,9 +1749,6 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1750,9 +1761,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1834,9 +1842,6 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1858,9 +1863,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1942,15 +1944,6 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="31" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1981,12 +1974,6 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="19" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2034,12 +2021,74 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="47">
+  <dxfs count="50">
+    <dxf>
+      <font>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF274E13"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2754,7 +2803,7 @@
     <col min="2" max="2" width="9" style="2" customWidth="1"/>
     <col min="3" max="3" width="22" style="6" customWidth="1"/>
     <col min="4" max="4" width="25" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.46484375" style="2" customWidth="1"/>
     <col min="6" max="6" width="10" style="2" customWidth="1"/>
     <col min="7" max="7" width="56" style="3" customWidth="1"/>
     <col min="8" max="8" width="14" style="3" customWidth="1"/>
@@ -2764,18 +2813,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="14" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="112" t="s">
         <v>344</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
+      <c r="B1" s="112"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
     </row>
     <row r="2" spans="1:17" s="16" customFormat="1" ht="24.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="15" t="s">
@@ -2810,34 +2859,34 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="29">
+      <c r="A3" s="28">
         <v>1</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="119" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="34" t="s">
+      <c r="F3" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="35" t="s">
+      <c r="G3" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="49" t="s">
+      <c r="H3" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="36" t="s">
+      <c r="J3" s="34" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2854,7 +2903,7 @@
       <c r="D4" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="125" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="22" t="s">
@@ -2863,7 +2912,7 @@
       <c r="G4" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="50" t="s">
+      <c r="H4" s="48" t="s">
         <v>16</v>
       </c>
       <c r="I4" s="24" t="s">
@@ -2886,7 +2935,7 @@
       <c r="D5" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F5" s="22" t="s">
@@ -2895,7 +2944,7 @@
       <c r="G5" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="50" t="s">
+      <c r="H5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="I5" s="24" t="s">
@@ -2918,7 +2967,7 @@
       <c r="D6" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="28" t="s">
+      <c r="E6" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F6" s="22" t="s">
@@ -2927,7 +2976,7 @@
       <c r="G6" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="50" t="s">
+      <c r="H6" s="48" t="s">
         <v>16</v>
       </c>
       <c r="I6" s="24" t="s">
@@ -2950,7 +2999,7 @@
       <c r="D7" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="22" t="s">
@@ -2959,7 +3008,7 @@
       <c r="G7" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="50" t="s">
+      <c r="H7" s="48" t="s">
         <v>16</v>
       </c>
       <c r="I7" s="24" t="s">
@@ -2982,16 +3031,16 @@
       <c r="D8" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="77" t="s">
+      <c r="G8" s="73" t="s">
         <v>44</v>
       </c>
-      <c r="H8" s="50" t="s">
+      <c r="H8" s="48" t="s">
         <v>16</v>
       </c>
       <c r="I8" s="24" t="s">
@@ -3014,7 +3063,7 @@
       <c r="D9" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F9" s="22" t="s">
@@ -3023,7 +3072,7 @@
       <c r="G9" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="50" t="s">
+      <c r="H9" s="48" t="s">
         <v>16</v>
       </c>
       <c r="I9" s="24" t="s">
@@ -3046,7 +3095,7 @@
       <c r="D10" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="22" t="s">
@@ -3055,7 +3104,7 @@
       <c r="G10" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="50" t="s">
+      <c r="H10" s="48" t="s">
         <v>16</v>
       </c>
       <c r="I10" s="24" t="s">
@@ -3078,7 +3127,7 @@
       <c r="D11" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="28" t="s">
+      <c r="E11" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="22" t="s">
@@ -3087,7 +3136,7 @@
       <c r="G11" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="H11" s="51" t="s">
+      <c r="H11" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I11" s="24" t="s">
@@ -3110,7 +3159,7 @@
       <c r="D12" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="22" t="s">
@@ -3119,7 +3168,7 @@
       <c r="G12" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="51" t="s">
+      <c r="H12" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I12" s="24" t="s">
@@ -3142,7 +3191,7 @@
       <c r="D13" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="E13" s="28" t="s">
+      <c r="E13" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F13" s="22" t="s">
@@ -3151,7 +3200,7 @@
       <c r="G13" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="H13" s="51" t="s">
+      <c r="H13" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I13" s="24" t="s">
@@ -3174,7 +3223,7 @@
       <c r="D14" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="28" t="s">
+      <c r="E14" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F14" s="22" t="s">
@@ -3183,7 +3232,7 @@
       <c r="G14" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="H14" s="51" t="s">
+      <c r="H14" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I14" s="24" t="s">
@@ -3206,16 +3255,16 @@
       <c r="D15" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E15" s="28" t="s">
+      <c r="E15" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F15" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="G15" s="62" t="s">
+      <c r="G15" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="H15" s="51" t="s">
+      <c r="H15" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I15" s="24" t="s">
@@ -3238,27 +3287,27 @@
       <c r="D16" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="28" t="s">
+      <c r="E16" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F16" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="G16" s="62" t="s">
+      <c r="G16" s="59" t="s">
         <v>86</v>
       </c>
-      <c r="H16" s="51" t="s">
+      <c r="H16" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I16" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="J16" s="75" t="s">
+      <c r="J16" s="71" t="s">
         <v>88</v>
       </c>
-      <c r="O16" s="78"/>
-      <c r="P16" s="78"/>
-      <c r="Q16" s="78"/>
+      <c r="O16" s="74"/>
+      <c r="P16" s="74"/>
+      <c r="Q16" s="74"/>
     </row>
     <row r="17" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="20">
@@ -3273,16 +3322,16 @@
       <c r="D17" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E17" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F17" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="G17" s="62" t="s">
+      <c r="G17" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="H17" s="51" t="s">
+      <c r="H17" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I17" s="24" t="s">
@@ -3291,12 +3340,12 @@
       <c r="J17" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="M17" s="51" t="s">
+      <c r="M17" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="O17" s="79"/>
-      <c r="P17" s="78"/>
-      <c r="Q17" s="79"/>
+      <c r="O17" s="75"/>
+      <c r="P17" s="74"/>
+      <c r="Q17" s="75"/>
     </row>
     <row r="18" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="20">
@@ -3311,16 +3360,16 @@
       <c r="D18" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="G18" s="62" t="s">
+      <c r="G18" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="51" t="s">
+      <c r="H18" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I18" s="24" t="s">
@@ -3329,9 +3378,9 @@
       <c r="J18" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="O18" s="78"/>
-      <c r="P18" s="78"/>
-      <c r="Q18" s="78"/>
+      <c r="O18" s="74"/>
+      <c r="P18" s="74"/>
+      <c r="Q18" s="74"/>
     </row>
     <row r="19" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="20">
@@ -3346,7 +3395,7 @@
       <c r="D19" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="28" t="s">
+      <c r="E19" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="22" t="s">
@@ -3355,7 +3404,7 @@
       <c r="G19" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="H19" s="51" t="s">
+      <c r="H19" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I19" s="24" t="s">
@@ -3364,7 +3413,7 @@
       <c r="J19" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="M19" s="51" t="s">
+      <c r="M19" s="49" t="s">
         <v>107</v>
       </c>
     </row>
@@ -3381,22 +3430,22 @@
       <c r="D20" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="E20" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="F20" s="83" t="s">
+      <c r="F20" s="79" t="s">
         <v>109</v>
       </c>
-      <c r="G20" s="82" t="s">
+      <c r="G20" s="78" t="s">
         <v>110</v>
       </c>
-      <c r="H20" s="51" t="s">
+      <c r="H20" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I20" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="J20" s="75" t="s">
+      <c r="J20" s="71" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3413,7 +3462,7 @@
       <c r="D21" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E21" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F21" s="22" t="s">
@@ -3422,7 +3471,7 @@
       <c r="G21" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="H21" s="51" t="s">
+      <c r="H21" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I21" s="24" t="s">
@@ -3431,7 +3480,7 @@
       <c r="J21" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="M21" s="51" t="s">
+      <c r="M21" s="49" t="s">
         <v>118</v>
       </c>
     </row>
@@ -3448,7 +3497,7 @@
       <c r="D22" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="E22" s="28" t="s">
+      <c r="E22" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F22" s="22" t="s">
@@ -3457,7 +3506,7 @@
       <c r="G22" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="H22" s="51" t="s">
+      <c r="H22" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I22" s="24" t="s">
@@ -3480,7 +3529,7 @@
       <c r="D23" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="120" t="s">
         <v>13</v>
       </c>
       <c r="F23" s="22" t="s">
@@ -3489,7 +3538,7 @@
       <c r="G23" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="H23" s="51" t="s">
+      <c r="H23" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I23" s="24" t="s">
@@ -3512,22 +3561,22 @@
       <c r="D24" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="E24" s="28" t="s">
+      <c r="E24" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="F24" s="102" t="s">
+      <c r="F24" s="95" t="s">
         <v>131</v>
       </c>
-      <c r="G24" s="101" t="s">
+      <c r="G24" s="94" t="s">
         <v>132</v>
       </c>
-      <c r="H24" s="51" t="s">
+      <c r="H24" s="49" t="s">
         <v>16</v>
       </c>
       <c r="I24" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="J24" s="84" t="s">
+      <c r="J24" s="80" t="s">
         <v>134</v>
       </c>
     </row>
@@ -3544,22 +3593,22 @@
       <c r="D25" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="E25" s="28" t="s">
+      <c r="E25" s="120" t="s">
         <v>136</v>
       </c>
-      <c r="F25" s="83" t="s">
+      <c r="F25" s="79" t="s">
         <v>137</v>
       </c>
       <c r="G25" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="H25" s="51" t="s">
+      <c r="H25" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I25" s="120" t="s">
+      <c r="I25" s="111" t="s">
         <v>139</v>
       </c>
-      <c r="J25" s="120" t="s">
+      <c r="J25" s="111" t="s">
         <v>140</v>
       </c>
     </row>
@@ -3576,310 +3625,310 @@
       <c r="D26" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="E26" s="28" t="s">
+      <c r="E26" s="120" t="s">
         <v>13</v>
       </c>
-      <c r="F26" s="83" t="s">
+      <c r="F26" s="79" t="s">
         <v>142</v>
       </c>
       <c r="G26" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="H26" s="51" t="s">
+      <c r="H26" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I26" s="120" t="s">
+      <c r="I26" s="111" t="s">
         <v>144</v>
       </c>
-      <c r="J26" s="120" t="s">
+      <c r="J26" s="111" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="56">
+      <c r="A27" s="54">
         <v>25</v>
       </c>
-      <c r="B27" s="58" t="s">
+      <c r="B27" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="C27" s="60" t="s">
+      <c r="C27" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D27" s="57" t="s">
+      <c r="D27" s="55" t="s">
         <v>146</v>
       </c>
       <c r="E27" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F27" s="126" t="s">
+      <c r="F27" s="117" t="s">
         <v>147</v>
       </c>
-      <c r="G27" s="127" t="s">
+      <c r="G27" s="118" t="s">
         <v>148</v>
       </c>
-      <c r="H27" s="51" t="s">
+      <c r="H27" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I27" s="125" t="s">
+      <c r="I27" s="116" t="s">
         <v>139</v>
       </c>
-      <c r="J27" s="125" t="s">
+      <c r="J27" s="116" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="56">
+      <c r="A28" s="54">
         <v>26</v>
       </c>
-      <c r="B28" s="58" t="s">
+      <c r="B28" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="C28" s="63" t="s">
+      <c r="C28" s="60" t="s">
         <v>150</v>
       </c>
-      <c r="D28" s="59" t="s">
+      <c r="D28" s="57" t="s">
         <v>151</v>
       </c>
-      <c r="E28" s="64" t="s">
+      <c r="E28" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F28" s="123" t="s">
+      <c r="F28" s="117" t="s">
         <v>152</v>
       </c>
-      <c r="G28" s="124" t="s">
+      <c r="G28" s="128" t="s">
         <v>153</v>
       </c>
-      <c r="H28" s="51" t="s">
-        <v>107</v>
-      </c>
-      <c r="I28" s="124" t="s">
+      <c r="H28" s="49" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="128" t="s">
         <v>154</v>
       </c>
-      <c r="J28" s="124" t="s">
+      <c r="J28" s="128" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="56">
+      <c r="A29" s="54">
         <v>27</v>
       </c>
-      <c r="B29" s="56" t="s">
+      <c r="B29" s="54" t="s">
         <v>95</v>
       </c>
-      <c r="C29" s="63" t="s">
+      <c r="C29" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="D29" s="59" t="s">
+      <c r="D29" s="57" t="s">
         <v>156</v>
       </c>
       <c r="E29" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="F29" s="58" t="s">
+      <c r="F29" s="56" t="s">
         <v>158</v>
       </c>
-      <c r="G29" s="76" t="s">
+      <c r="G29" s="72" t="s">
         <v>159</v>
       </c>
-      <c r="H29" s="51" t="s">
+      <c r="H29" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I29" s="59" t="s">
+      <c r="I29" s="57" t="s">
         <v>160</v>
       </c>
-      <c r="J29" s="59" t="s">
+      <c r="J29" s="57" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="30" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="56">
+      <c r="A30" s="54">
         <v>28</v>
       </c>
-      <c r="B30" s="56" t="s">
+      <c r="B30" s="54" t="s">
         <v>95</v>
       </c>
-      <c r="C30" s="63" t="s">
+      <c r="C30" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="59" t="s">
+      <c r="D30" s="57" t="s">
         <v>156</v>
       </c>
       <c r="E30" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="F30" s="58" t="s">
+      <c r="F30" s="114" t="s">
         <v>162</v>
       </c>
-      <c r="G30" s="59" t="s">
+      <c r="G30" s="115" t="s">
         <v>163</v>
       </c>
-      <c r="H30" s="57" t="s">
-        <v>118</v>
-      </c>
-      <c r="I30" s="59" t="s">
+      <c r="H30" s="49" t="s">
+        <v>107</v>
+      </c>
+      <c r="I30" s="115" t="s">
         <v>164</v>
       </c>
-      <c r="J30" s="59" t="s">
+      <c r="J30" s="115" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="56">
+      <c r="A31" s="54">
         <v>29</v>
       </c>
-      <c r="B31" s="56" t="s">
+      <c r="B31" s="54" t="s">
         <v>95</v>
       </c>
-      <c r="C31" s="63" t="s">
+      <c r="C31" s="60" t="s">
         <v>166</v>
       </c>
-      <c r="D31" s="59" t="s">
+      <c r="D31" s="57" t="s">
         <v>167</v>
       </c>
       <c r="E31" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F31" s="58" t="s">
+      <c r="F31" s="56" t="s">
         <v>168</v>
       </c>
-      <c r="G31" s="59" t="s">
+      <c r="G31" s="57" t="s">
         <v>169</v>
       </c>
-      <c r="H31" s="57" t="s">
+      <c r="H31" s="55" t="s">
         <v>118</v>
       </c>
-      <c r="I31" s="59" t="s">
+      <c r="I31" s="57" t="s">
         <v>170</v>
       </c>
-      <c r="J31" s="59" t="s">
+      <c r="J31" s="57" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="56">
+      <c r="A32" s="54">
         <v>30</v>
       </c>
-      <c r="B32" s="56" t="s">
+      <c r="B32" s="54" t="s">
         <v>95</v>
       </c>
-      <c r="C32" s="63" t="s">
+      <c r="C32" s="60" t="s">
         <v>172</v>
       </c>
-      <c r="D32" s="59" t="s">
+      <c r="D32" s="57" t="s">
         <v>173</v>
       </c>
       <c r="E32" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F32" s="58" t="s">
+      <c r="F32" s="56" t="s">
         <v>174</v>
       </c>
-      <c r="G32" s="59" t="s">
+      <c r="G32" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="H32" s="57" t="s">
+      <c r="H32" s="55" t="s">
         <v>118</v>
       </c>
-      <c r="I32" s="59" t="s">
+      <c r="I32" s="57" t="s">
         <v>160</v>
       </c>
-      <c r="J32" s="59" t="s">
+      <c r="J32" s="57" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="56">
+      <c r="A33" s="54">
         <v>31</v>
       </c>
-      <c r="B33" s="56" t="s">
+      <c r="B33" s="54" t="s">
         <v>95</v>
       </c>
-      <c r="C33" s="63" t="s">
+      <c r="C33" s="60" t="s">
         <v>177</v>
       </c>
-      <c r="D33" s="59" t="s">
+      <c r="D33" s="57" t="s">
         <v>178</v>
       </c>
       <c r="E33" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F33" s="80" t="s">
+      <c r="F33" s="76" t="s">
         <v>179</v>
       </c>
-      <c r="G33" s="100" t="s">
+      <c r="G33" s="93" t="s">
         <v>180</v>
       </c>
-      <c r="H33" s="57" t="s">
+      <c r="H33" s="55" t="s">
         <v>107</v>
       </c>
-      <c r="I33" s="100" t="s">
+      <c r="I33" s="93" t="s">
         <v>181</v>
       </c>
-      <c r="J33" s="100" t="s">
+      <c r="J33" s="93" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="56">
+      <c r="A34" s="54">
         <v>32</v>
       </c>
-      <c r="B34" s="112" t="s">
+      <c r="B34" s="103" t="s">
         <v>95</v>
       </c>
-      <c r="C34" s="63" t="s">
+      <c r="C34" s="60" t="s">
         <v>177</v>
       </c>
-      <c r="D34" s="59" t="s">
+      <c r="D34" s="57" t="s">
         <v>183</v>
       </c>
       <c r="E34" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F34" s="58" t="s">
+      <c r="F34" s="56" t="s">
         <v>184</v>
       </c>
-      <c r="G34" s="59" t="s">
+      <c r="G34" s="57" t="s">
         <v>185</v>
       </c>
-      <c r="H34" s="57" t="s">
+      <c r="H34" s="55" t="s">
         <v>118</v>
       </c>
-      <c r="I34" s="59" t="s">
+      <c r="I34" s="57" t="s">
         <v>186</v>
       </c>
-      <c r="J34" s="59" t="s">
+      <c r="J34" s="57" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="35" spans="1:13" s="10" customFormat="1" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="66">
+    <row r="35" spans="1:13" s="10" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="63">
         <v>33</v>
       </c>
-      <c r="B35" s="113" t="s">
+      <c r="B35" s="104" t="s">
         <v>95</v>
       </c>
-      <c r="C35" s="95" t="s">
+      <c r="C35" s="91" t="s">
         <v>172</v>
       </c>
-      <c r="D35" s="68" t="s">
+      <c r="D35" s="65" t="s">
         <v>188</v>
       </c>
-      <c r="E35" s="69" t="s">
+      <c r="E35" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="F35" s="73" t="s">
+      <c r="F35" s="69" t="s">
         <v>189</v>
       </c>
-      <c r="G35" s="90" t="s">
+      <c r="G35" s="86" t="s">
         <v>190</v>
       </c>
       <c r="H35" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="I35" s="81" t="s">
+      <c r="I35" s="77" t="s">
         <v>191</v>
       </c>
-      <c r="J35" s="81" t="s">
+      <c r="J35" s="77" t="s">
         <v>192</v>
       </c>
       <c r="K35"/>
@@ -3887,34 +3936,34 @@
       <c r="M35"/>
     </row>
     <row r="36" spans="1:13" s="10" customFormat="1" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="66">
+      <c r="A36" s="63">
         <v>34</v>
       </c>
-      <c r="B36" s="67" t="s">
+      <c r="B36" s="64" t="s">
         <v>193</v>
       </c>
-      <c r="C36" s="71" t="s">
+      <c r="C36" s="67" t="s">
         <v>194</v>
       </c>
-      <c r="D36" s="68" t="s">
+      <c r="D36" s="65" t="s">
         <v>195</v>
       </c>
-      <c r="E36" s="69" t="s">
+      <c r="E36" s="121" t="s">
         <v>13</v>
       </c>
-      <c r="F36" s="73" t="s">
+      <c r="F36" s="69" t="s">
         <v>196</v>
       </c>
-      <c r="G36" s="68" t="s">
+      <c r="G36" s="65" t="s">
         <v>197</v>
       </c>
-      <c r="H36" s="57" t="s">
+      <c r="H36" s="55" t="s">
         <v>118</v>
       </c>
-      <c r="I36" s="68" t="s">
+      <c r="I36" s="65" t="s">
         <v>198</v>
       </c>
-      <c r="J36" s="68" t="s">
+      <c r="J36" s="65" t="s">
         <v>199</v>
       </c>
       <c r="K36"/>
@@ -3922,28 +3971,28 @@
       <c r="M36"/>
     </row>
     <row r="37" spans="1:13" s="10" customFormat="1" ht="14.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A37" s="70">
+      <c r="A37" s="66">
         <v>35</v>
       </c>
-      <c r="B37" s="93" t="s">
+      <c r="B37" s="89" t="s">
         <v>193</v>
       </c>
-      <c r="C37" s="72" t="s">
+      <c r="C37" s="68" t="s">
         <v>200</v>
       </c>
       <c r="D37" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="E37" s="97" t="s">
+      <c r="E37" s="126" t="s">
         <v>202</v>
       </c>
-      <c r="F37" s="74" t="s">
+      <c r="F37" s="70" t="s">
         <v>203</v>
       </c>
       <c r="G37" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="H37" s="65" t="s">
+      <c r="H37" s="62" t="s">
         <v>118</v>
       </c>
       <c r="I37" s="10" t="s">
@@ -3957,34 +4006,34 @@
       <c r="M37"/>
     </row>
     <row r="38" spans="1:13" ht="14.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A38" s="88">
+      <c r="A38" s="84">
         <v>36</v>
       </c>
-      <c r="B38" s="117" t="s">
+      <c r="B38" s="108" t="s">
         <v>207</v>
       </c>
-      <c r="C38" s="96" t="s">
+      <c r="C38" s="92" t="s">
         <v>11</v>
       </c>
-      <c r="D38" s="87" t="s">
+      <c r="D38" s="83" t="s">
         <v>208</v>
       </c>
-      <c r="E38" s="98" t="s">
+      <c r="E38" s="127" t="s">
         <v>209</v>
       </c>
-      <c r="F38" s="91" t="s">
+      <c r="F38" s="87" t="s">
         <v>210</v>
       </c>
-      <c r="G38" s="92" t="s">
+      <c r="G38" s="88" t="s">
         <v>345</v>
       </c>
-      <c r="H38" s="85" t="s">
+      <c r="H38" s="81" t="s">
         <v>118</v>
       </c>
-      <c r="I38" s="87" t="s">
+      <c r="I38" s="83" t="s">
         <v>211</v>
       </c>
-      <c r="J38" s="87" t="s">
+      <c r="J38" s="83" t="s">
         <v>212</v>
       </c>
       <c r="K38"/>
@@ -3992,34 +4041,34 @@
       <c r="M38"/>
     </row>
     <row r="39" spans="1:13" ht="14.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A39" s="88">
+      <c r="A39" s="84">
         <v>37</v>
       </c>
-      <c r="B39" s="114" t="s">
+      <c r="B39" s="105" t="s">
         <v>95</v>
       </c>
-      <c r="C39" s="96" t="s">
+      <c r="C39" s="92" t="s">
         <v>177</v>
       </c>
-      <c r="D39" s="87" t="s">
+      <c r="D39" s="83" t="s">
         <v>213</v>
       </c>
-      <c r="E39" s="98" t="s">
+      <c r="E39" s="122" t="s">
         <v>214</v>
       </c>
-      <c r="F39" s="91" t="s">
+      <c r="F39" s="87" t="s">
         <v>215</v>
       </c>
-      <c r="G39" s="87" t="s">
+      <c r="G39" s="83" t="s">
         <v>216</v>
       </c>
-      <c r="H39" s="85" t="s">
+      <c r="H39" s="81" t="s">
         <v>118</v>
       </c>
-      <c r="I39" s="87" t="s">
+      <c r="I39" s="83" t="s">
         <v>217</v>
       </c>
-      <c r="J39" s="87" t="s">
+      <c r="J39" s="83" t="s">
         <v>218</v>
       </c>
       <c r="K39"/>
@@ -4027,34 +4076,34 @@
       <c r="M39"/>
     </row>
     <row r="40" spans="1:13" ht="14.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A40" s="88">
+      <c r="A40" s="84">
         <v>38</v>
       </c>
-      <c r="B40" s="94" t="s">
+      <c r="B40" s="90" t="s">
         <v>193</v>
       </c>
-      <c r="C40" s="96" t="s">
+      <c r="C40" s="92" t="s">
         <v>219</v>
       </c>
-      <c r="D40" s="87" t="s">
+      <c r="D40" s="83" t="s">
         <v>220</v>
       </c>
-      <c r="E40" s="99" t="s">
+      <c r="E40" s="122" t="s">
         <v>221</v>
       </c>
-      <c r="F40" s="91" t="s">
+      <c r="F40" s="87" t="s">
         <v>222</v>
       </c>
-      <c r="G40" s="87" t="s">
+      <c r="G40" s="83" t="s">
         <v>223</v>
       </c>
-      <c r="H40" s="85" t="s">
+      <c r="H40" s="81" t="s">
         <v>118</v>
       </c>
-      <c r="I40" s="87" t="s">
+      <c r="I40" s="83" t="s">
         <v>160</v>
       </c>
-      <c r="J40" s="87" t="s">
+      <c r="J40" s="83" t="s">
         <v>224</v>
       </c>
       <c r="K40"/>
@@ -4062,34 +4111,34 @@
       <c r="M40"/>
     </row>
     <row r="41" spans="1:13" ht="14.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A41" s="106">
+      <c r="A41" s="99">
         <v>39</v>
       </c>
-      <c r="B41" s="115" t="s">
+      <c r="B41" s="106" t="s">
         <v>95</v>
       </c>
-      <c r="C41" s="118" t="s">
+      <c r="C41" s="109" t="s">
         <v>25</v>
       </c>
-      <c r="D41" s="105" t="s">
+      <c r="D41" s="98" t="s">
         <v>225</v>
       </c>
-      <c r="E41" s="110" t="s">
+      <c r="E41" s="123" t="s">
         <v>27</v>
       </c>
-      <c r="F41" s="108" t="s">
+      <c r="F41" s="101" t="s">
         <v>226</v>
       </c>
-      <c r="G41" s="109" t="s">
+      <c r="G41" s="102" t="s">
         <v>227</v>
       </c>
-      <c r="H41" s="103" t="s">
+      <c r="H41" s="96" t="s">
         <v>118</v>
       </c>
-      <c r="I41" s="105" t="s">
+      <c r="I41" s="98" t="s">
         <v>228</v>
       </c>
-      <c r="J41" s="105" t="s">
+      <c r="J41" s="98" t="s">
         <v>229</v>
       </c>
       <c r="K41"/>
@@ -4097,28 +4146,28 @@
       <c r="M41"/>
     </row>
     <row r="42" spans="1:13" ht="14.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="89">
+      <c r="A42" s="85">
         <v>40</v>
       </c>
-      <c r="B42" s="116" t="s">
+      <c r="B42" s="107" t="s">
         <v>95</v>
       </c>
-      <c r="C42" s="119" t="s">
+      <c r="C42" s="110" t="s">
         <v>338</v>
       </c>
       <c r="D42" s="13" t="s">
         <v>339</v>
       </c>
-      <c r="E42" s="111" t="s">
+      <c r="E42" s="124" t="s">
         <v>27</v>
       </c>
-      <c r="F42" s="107" t="s">
+      <c r="F42" s="100" t="s">
         <v>340</v>
       </c>
       <c r="G42" s="13" t="s">
         <v>341</v>
       </c>
-      <c r="H42" s="104" t="s">
+      <c r="H42" s="97" t="s">
         <v>118</v>
       </c>
       <c r="I42" s="13" t="s">
@@ -4132,14 +4181,14 @@
       <c r="M42"/>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A43" s="89"/>
-      <c r="B43" s="89"/>
+      <c r="A43" s="85"/>
+      <c r="B43" s="85"/>
       <c r="C43" s="13"/>
       <c r="D43" s="13"/>
-      <c r="E43" s="89"/>
-      <c r="F43" s="89"/>
+      <c r="E43" s="85"/>
+      <c r="F43" s="85"/>
       <c r="G43" s="13"/>
-      <c r="H43" s="86"/>
+      <c r="H43" s="82"/>
       <c r="I43" s="13"/>
       <c r="J43" s="13"/>
     </row>
@@ -4192,147 +4241,156 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B27">
-    <cfRule type="expression" dxfId="46" priority="41">
+    <cfRule type="expression" dxfId="49" priority="44">
       <formula>B3="P0"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="42">
+    <cfRule type="expression" dxfId="48" priority="45">
       <formula>B3="P1"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="43">
+    <cfRule type="expression" dxfId="47" priority="46">
       <formula>B3="P2"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="44">
+    <cfRule type="expression" dxfId="46" priority="47">
       <formula>B3="P3"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B34">
-    <cfRule type="expression" dxfId="42" priority="46">
+    <cfRule type="expression" dxfId="45" priority="49">
       <formula>B3="P1"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="45">
+    <cfRule type="expression" dxfId="44" priority="48">
       <formula>B3="P0"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="47">
+    <cfRule type="expression" dxfId="43" priority="50">
       <formula>B3="P2"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="48">
+    <cfRule type="expression" dxfId="42" priority="51">
       <formula>B3="P3"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H28">
-    <cfRule type="expression" dxfId="38" priority="39">
+    <cfRule type="expression" dxfId="41" priority="42">
       <formula>H3="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="38">
+    <cfRule type="expression" dxfId="40" priority="41">
       <formula>H3="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="40">
+    <cfRule type="expression" dxfId="39" priority="43">
       <formula>H3="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="35" priority="49">
+    <cfRule type="expression" dxfId="38" priority="52">
       <formula>H3="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="50">
+    <cfRule type="expression" dxfId="37" priority="53">
       <formula>H3="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="51">
+    <cfRule type="expression" dxfId="36" priority="54">
       <formula>H3="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H29">
-    <cfRule type="expression" dxfId="32" priority="33">
+    <cfRule type="expression" dxfId="35" priority="36">
       <formula>H29="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="32">
+    <cfRule type="expression" dxfId="34" priority="35">
       <formula>H29="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="31">
+    <cfRule type="expression" dxfId="33" priority="34">
       <formula>H29="Completed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M17">
+    <cfRule type="expression" dxfId="32" priority="32">
+      <formula>M17="In Process"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="31" priority="31">
+      <formula>M17="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="30" priority="30">
+      <formula>M17="Not Started"</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="29" priority="29">
       <formula>M17="In Process"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="28" priority="28">
       <formula>M17="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="27">
-      <formula>M17="Not Started"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="26" priority="26">
-      <formula>M17="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="25" priority="25">
-      <formula>M17="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="30">
+    <cfRule type="expression" dxfId="27" priority="33">
       <formula>M17="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M19">
-    <cfRule type="expression" dxfId="23" priority="11">
+    <cfRule type="expression" dxfId="26" priority="14">
       <formula>M19="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="7">
+    <cfRule type="expression" dxfId="25" priority="10">
       <formula>M19="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="8">
+    <cfRule type="expression" dxfId="24" priority="11">
       <formula>M19="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="9">
+    <cfRule type="expression" dxfId="23" priority="12">
       <formula>M19="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="10">
+    <cfRule type="expression" dxfId="22" priority="13">
       <formula>M19="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="12">
+    <cfRule type="expression" dxfId="21" priority="15">
       <formula>M19="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M21">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="20" priority="4">
       <formula>M21="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="19" priority="5">
       <formula>M21="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="18" priority="6">
       <formula>M21="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="17" priority="7">
       <formula>M21="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="16" priority="8">
       <formula>M21="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="15" priority="9">
       <formula>M21="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O17">
+    <cfRule type="expression" dxfId="14" priority="26">
+      <formula>O17="In Process"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="25">
+      <formula>O17="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="24">
+      <formula>O17="Not Started"</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="11" priority="23">
       <formula>O17="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="22">
-      <formula>O17="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="21">
+    <cfRule type="expression" dxfId="10" priority="27">
       <formula>O17="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="20">
-      <formula>O17="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="24">
-      <formula>O17="Not Started"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="19">
+    <cfRule type="expression" dxfId="9" priority="22">
       <formula>O17="Completed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q17">
+    <cfRule type="expression" dxfId="8" priority="21">
+      <formula>Q17="Not Started"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="20">
+      <formula>Q17="In Process"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="19">
+      <formula>Q17="Completed"</formula>
+    </cfRule>
     <cfRule type="expression" dxfId="5" priority="18">
       <formula>Q17="Not Started"</formula>
     </cfRule>
@@ -4342,14 +4400,16 @@
     <cfRule type="expression" dxfId="3" priority="16">
       <formula>Q17="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="15">
-      <formula>Q17="Not Started"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>H30="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="14">
-      <formula>Q17="In Process"</formula>
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>H30="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="13">
-      <formula>Q17="Completed"</formula>
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>H30="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -4380,14 +4440,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="8" customFormat="1" ht="0.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="122" t="s">
+      <c r="A1" s="113" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="122"/>
-      <c r="C1" s="122"/>
-      <c r="D1" s="122"/>
-      <c r="E1" s="122"/>
-      <c r="F1" s="122"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
     </row>
     <row r="2" spans="1:6" ht="0.2" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4"/>
@@ -4415,7 +4475,7 @@
       <c r="A4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="50" t="s">
         <v>233</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -4429,7 +4489,7 @@
       <c r="A5" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="51" t="s">
         <v>235</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -4443,7 +4503,7 @@
       <c r="A6" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="52" t="s">
         <v>237</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -4457,7 +4517,7 @@
       <c r="A7" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="53" t="s">
         <v>239</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -4490,13 +4550,13 @@
       <c r="F9" s="13"/>
     </row>
     <row r="10" spans="1:6" ht="0.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="47" t="s">
+      <c r="A10" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="48" t="s">
+      <c r="B10" s="46" t="s">
         <v>242</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="46" t="s">
         <v>243</v>
       </c>
       <c r="D10" s="7"/>
@@ -4755,13 +4815,13 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="0.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="37" t="s">
+      <c r="A30" s="35" t="s">
         <v>289</v>
       </c>
-      <c r="B30" s="37" t="s">
+      <c r="B30" s="35" t="s">
         <v>290</v>
       </c>
-      <c r="C30" s="37" t="s">
+      <c r="C30" s="35" t="s">
         <v>291</v>
       </c>
     </row>
@@ -4773,84 +4833,84 @@
       <c r="C31" s="13"/>
     </row>
     <row r="32" spans="1:6" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="38"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
+      <c r="A32" s="36"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
     </row>
     <row r="33" spans="1:3" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="39" t="s">
+      <c r="A33" s="37" t="s">
         <v>293</v>
       </c>
-      <c r="B33" s="40" t="s">
+      <c r="B33" s="38" t="s">
         <v>294</v>
       </c>
-      <c r="C33" s="41" t="s">
+      <c r="C33" s="39" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="42" t="s">
+      <c r="A34" s="40" t="s">
         <v>296</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="C34" s="43" t="s">
+      <c r="C34" s="41" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="42" t="s">
+      <c r="A35" s="40" t="s">
         <v>299</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="C35" s="43" t="s">
+      <c r="C35" s="41" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="42" t="s">
+      <c r="A36" s="40" t="s">
         <v>302</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C36" s="43" t="s">
+      <c r="C36" s="41" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="42" t="s">
+      <c r="A37" s="40" t="s">
         <v>305</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="C37" s="43" t="s">
+      <c r="C37" s="41" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="42" t="s">
+      <c r="A38" s="40" t="s">
         <v>308</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="C38" s="43" t="s">
+      <c r="C38" s="41" t="s">
         <v>310</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="0.3" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="44" t="s">
+      <c r="A39" s="42" t="s">
         <v>311</v>
       </c>
-      <c r="B39" s="45" t="s">
+      <c r="B39" s="43" t="s">
         <v>312</v>
       </c>
-      <c r="C39" s="46" t="s">
+      <c r="C39" s="44" t="s">
         <v>313</v>
       </c>
     </row>
@@ -4877,13 +4937,13 @@
       </c>
     </row>
     <row r="42" spans="1:3" ht="0.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="37" t="s">
+      <c r="A42" s="35" t="s">
         <v>319</v>
       </c>
-      <c r="B42" s="37" t="s">
+      <c r="B42" s="35" t="s">
         <v>320</v>
       </c>
-      <c r="C42" s="37" t="s">
+      <c r="C42" s="35" t="s">
         <v>321</v>
       </c>
     </row>
@@ -4895,51 +4955,51 @@
       <c r="C43" s="13"/>
     </row>
     <row r="44" spans="1:3" ht="0.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A44" s="38"/>
-      <c r="B44" s="38"/>
-      <c r="C44" s="38"/>
+      <c r="A44" s="36"/>
+      <c r="B44" s="36"/>
+      <c r="C44" s="36"/>
     </row>
     <row r="45" spans="1:3" ht="0.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A45" s="39" t="s">
+      <c r="A45" s="37" t="s">
         <v>323</v>
       </c>
-      <c r="B45" s="40" t="s">
+      <c r="B45" s="38" t="s">
         <v>324</v>
       </c>
-      <c r="C45" s="41" t="s">
+      <c r="C45" s="39" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="0.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="42" t="s">
+      <c r="A46" s="40" t="s">
         <v>326</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="C46" s="43" t="s">
+      <c r="C46" s="41" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="0.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="42" t="s">
+      <c r="A47" s="40" t="s">
         <v>329</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="C47" s="43" t="s">
+      <c r="C47" s="41" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="0.4" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A48" s="44" t="s">
+      <c r="A48" s="42" t="s">
         <v>332</v>
       </c>
-      <c r="B48" s="45" t="s">
+      <c r="B48" s="43" t="s">
         <v>333</v>
       </c>
-      <c r="C48" s="46" t="s">
+      <c r="C48" s="44" t="s">
         <v>334</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated documents in support I-20 implementation tasks.
</commit_message>
<xml_diff>
--- a/planing/implementation-plan/azure-policy-assist-prioritized-implementation-log-v12.xlsx
+++ b/planing/implementation-plan/azure-policy-assist-prioritized-implementation-log-v12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steven\GitHub-Repositories\Repositories\azure-policy-assistant-rag-solution-docs\planing\implementation-plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{745A0F1F-4CB1-4E77-BFF2-63B2EC617C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F97FA7E2-C76F-468D-AC28-8B8E86D70550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="14235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Policy Implementation Backlog" sheetId="1" r:id="rId1"/>
@@ -2001,53 +2001,53 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="23" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2056,7 +2056,29 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="50">
+  <dxfs count="44">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF274E13"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF990000"/>
@@ -2064,6 +2086,223 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF38761D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF274E13"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF38761D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF274E13"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF38761D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF38761D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF990000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2135,17 +2374,6 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
         <color rgb="FF990000"/>
       </font>
       <fill>
@@ -2157,38 +2385,6 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF990000"/>
       </font>
       <fill>
@@ -2216,39 +2412,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF38761D"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2287,7 +2450,6 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF990000"/>
       </font>
       <fill>
         <patternFill>
@@ -2298,212 +2460,16 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF38761D"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFFCE5CD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF38761D"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF38761D"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF990000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF274E13"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
       </font>
       <fill>
         <patternFill>
@@ -2518,16 +2484,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2554,34 +2510,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCE5CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2813,18 +2749,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="14" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="125" t="s">
         <v>344</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="112"/>
-      <c r="J1" s="112"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="125"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
+      <c r="F1" s="125"/>
+      <c r="G1" s="125"/>
+      <c r="H1" s="125"/>
+      <c r="I1" s="125"/>
+      <c r="J1" s="125"/>
     </row>
     <row r="2" spans="1:17" s="16" customFormat="1" ht="24.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="15" t="s">
@@ -2871,7 +2807,7 @@
       <c r="D3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="119" t="s">
+      <c r="E3" s="115" t="s">
         <v>13</v>
       </c>
       <c r="F3" s="32" t="s">
@@ -2903,7 +2839,7 @@
       <c r="D4" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="125" t="s">
+      <c r="E4" s="121" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="22" t="s">
@@ -2935,7 +2871,7 @@
       <c r="D5" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="120" t="s">
+      <c r="E5" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F5" s="22" t="s">
@@ -2967,7 +2903,7 @@
       <c r="D6" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="120" t="s">
+      <c r="E6" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F6" s="22" t="s">
@@ -2999,7 +2935,7 @@
       <c r="D7" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="120" t="s">
+      <c r="E7" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="22" t="s">
@@ -3031,7 +2967,7 @@
       <c r="D8" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="120" t="s">
+      <c r="E8" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="22" t="s">
@@ -3063,7 +2999,7 @@
       <c r="D9" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="120" t="s">
+      <c r="E9" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F9" s="22" t="s">
@@ -3095,7 +3031,7 @@
       <c r="D10" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="120" t="s">
+      <c r="E10" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="22" t="s">
@@ -3127,7 +3063,7 @@
       <c r="D11" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="120" t="s">
+      <c r="E11" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="22" t="s">
@@ -3159,7 +3095,7 @@
       <c r="D12" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="120" t="s">
+      <c r="E12" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="22" t="s">
@@ -3191,7 +3127,7 @@
       <c r="D13" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="E13" s="120" t="s">
+      <c r="E13" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F13" s="22" t="s">
@@ -3223,7 +3159,7 @@
       <c r="D14" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="120" t="s">
+      <c r="E14" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F14" s="22" t="s">
@@ -3255,7 +3191,7 @@
       <c r="D15" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E15" s="120" t="s">
+      <c r="E15" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F15" s="22" t="s">
@@ -3287,7 +3223,7 @@
       <c r="D16" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="120" t="s">
+      <c r="E16" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F16" s="22" t="s">
@@ -3322,7 +3258,7 @@
       <c r="D17" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="E17" s="120" t="s">
+      <c r="E17" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F17" s="22" t="s">
@@ -3360,7 +3296,7 @@
       <c r="D18" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="120" t="s">
+      <c r="E18" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="22" t="s">
@@ -3395,7 +3331,7 @@
       <c r="D19" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="120" t="s">
+      <c r="E19" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="22" t="s">
@@ -3430,7 +3366,7 @@
       <c r="D20" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="E20" s="120" t="s">
+      <c r="E20" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F20" s="79" t="s">
@@ -3462,7 +3398,7 @@
       <c r="D21" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="120" t="s">
+      <c r="E21" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F21" s="22" t="s">
@@ -3497,7 +3433,7 @@
       <c r="D22" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="E22" s="120" t="s">
+      <c r="E22" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F22" s="22" t="s">
@@ -3529,7 +3465,7 @@
       <c r="D23" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="E23" s="120" t="s">
+      <c r="E23" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F23" s="22" t="s">
@@ -3561,7 +3497,7 @@
       <c r="D24" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="E24" s="120" t="s">
+      <c r="E24" s="116" t="s">
         <v>27</v>
       </c>
       <c r="F24" s="95" t="s">
@@ -3593,7 +3529,7 @@
       <c r="D25" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="E25" s="120" t="s">
+      <c r="E25" s="116" t="s">
         <v>136</v>
       </c>
       <c r="F25" s="79" t="s">
@@ -3625,7 +3561,7 @@
       <c r="D26" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="E26" s="120" t="s">
+      <c r="E26" s="116" t="s">
         <v>13</v>
       </c>
       <c r="F26" s="79" t="s">
@@ -3660,19 +3596,19 @@
       <c r="E27" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F27" s="117" t="s">
+      <c r="F27" s="114" t="s">
         <v>147</v>
       </c>
-      <c r="G27" s="118" t="s">
+      <c r="G27" s="23" t="s">
         <v>148</v>
       </c>
       <c r="H27" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I27" s="116" t="s">
+      <c r="I27" s="111" t="s">
         <v>139</v>
       </c>
-      <c r="J27" s="116" t="s">
+      <c r="J27" s="111" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3692,19 +3628,19 @@
       <c r="E28" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F28" s="117" t="s">
+      <c r="F28" s="114" t="s">
         <v>152</v>
       </c>
-      <c r="G28" s="128" t="s">
+      <c r="G28" s="124" t="s">
         <v>153</v>
       </c>
       <c r="H28" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="I28" s="128" t="s">
+      <c r="I28" s="124" t="s">
         <v>154</v>
       </c>
-      <c r="J28" s="128" t="s">
+      <c r="J28" s="124" t="s">
         <v>155</v>
       </c>
     </row>
@@ -3756,19 +3692,19 @@
       <c r="E30" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="F30" s="114" t="s">
+      <c r="F30" s="127" t="s">
         <v>162</v>
       </c>
-      <c r="G30" s="115" t="s">
+      <c r="G30" s="128" t="s">
         <v>163</v>
       </c>
       <c r="H30" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="I30" s="115" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" s="128" t="s">
         <v>164</v>
       </c>
-      <c r="J30" s="115" t="s">
+      <c r="J30" s="128" t="s">
         <v>165</v>
       </c>
     </row>
@@ -3788,19 +3724,19 @@
       <c r="E31" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F31" s="56" t="s">
+      <c r="F31" s="112" t="s">
         <v>168</v>
       </c>
-      <c r="G31" s="57" t="s">
+      <c r="G31" s="113" t="s">
         <v>169</v>
       </c>
-      <c r="H31" s="55" t="s">
-        <v>118</v>
-      </c>
-      <c r="I31" s="57" t="s">
+      <c r="H31" s="49" t="s">
+        <v>107</v>
+      </c>
+      <c r="I31" s="113" t="s">
         <v>170</v>
       </c>
-      <c r="J31" s="57" t="s">
+      <c r="J31" s="113" t="s">
         <v>171</v>
       </c>
     </row>
@@ -3913,7 +3849,7 @@
       <c r="D35" s="65" t="s">
         <v>188</v>
       </c>
-      <c r="E35" s="121" t="s">
+      <c r="E35" s="117" t="s">
         <v>27</v>
       </c>
       <c r="F35" s="69" t="s">
@@ -3948,7 +3884,7 @@
       <c r="D36" s="65" t="s">
         <v>195</v>
       </c>
-      <c r="E36" s="121" t="s">
+      <c r="E36" s="117" t="s">
         <v>13</v>
       </c>
       <c r="F36" s="69" t="s">
@@ -3983,7 +3919,7 @@
       <c r="D37" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="E37" s="126" t="s">
+      <c r="E37" s="122" t="s">
         <v>202</v>
       </c>
       <c r="F37" s="70" t="s">
@@ -4018,7 +3954,7 @@
       <c r="D38" s="83" t="s">
         <v>208</v>
       </c>
-      <c r="E38" s="127" t="s">
+      <c r="E38" s="123" t="s">
         <v>209</v>
       </c>
       <c r="F38" s="87" t="s">
@@ -4053,7 +3989,7 @@
       <c r="D39" s="83" t="s">
         <v>213</v>
       </c>
-      <c r="E39" s="122" t="s">
+      <c r="E39" s="118" t="s">
         <v>214</v>
       </c>
       <c r="F39" s="87" t="s">
@@ -4088,7 +4024,7 @@
       <c r="D40" s="83" t="s">
         <v>220</v>
       </c>
-      <c r="E40" s="122" t="s">
+      <c r="E40" s="118" t="s">
         <v>221</v>
       </c>
       <c r="F40" s="87" t="s">
@@ -4123,7 +4059,7 @@
       <c r="D41" s="98" t="s">
         <v>225</v>
       </c>
-      <c r="E41" s="123" t="s">
+      <c r="E41" s="119" t="s">
         <v>27</v>
       </c>
       <c r="F41" s="101" t="s">
@@ -4158,7 +4094,7 @@
       <c r="D42" s="13" t="s">
         <v>339</v>
       </c>
-      <c r="E42" s="124" t="s">
+      <c r="E42" s="120" t="s">
         <v>27</v>
       </c>
       <c r="F42" s="100" t="s">
@@ -4241,175 +4177,153 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:B27">
-    <cfRule type="expression" dxfId="49" priority="44">
-      <formula>B3="P0"</formula>
+    <cfRule type="expression" dxfId="43" priority="47">
+      <formula>B3="P3"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="45">
+    <cfRule type="expression" dxfId="42" priority="46">
+      <formula>B3="P2"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="41" priority="45">
       <formula>B3="P1"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="46">
-      <formula>B3="P2"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="46" priority="47">
-      <formula>B3="P3"</formula>
+    <cfRule type="expression" dxfId="40" priority="44">
+      <formula>B3="P0"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B34">
-    <cfRule type="expression" dxfId="45" priority="49">
+    <cfRule type="expression" dxfId="39" priority="51">
+      <formula>B3="P3"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="38" priority="50">
+      <formula>B3="P2"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="37" priority="49">
       <formula>B3="P1"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="48">
+    <cfRule type="expression" dxfId="36" priority="48">
       <formula>B3="P0"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="50">
-      <formula>B3="P2"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H31">
+    <cfRule type="expression" dxfId="35" priority="1">
+      <formula>H3="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="51">
-      <formula>B3="P3"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H28">
-    <cfRule type="expression" dxfId="41" priority="42">
+    <cfRule type="expression" dxfId="34" priority="2">
       <formula>H3="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="41">
-      <formula>H3="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="39" priority="43">
+    <cfRule type="expression" dxfId="33" priority="3">
       <formula>H3="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="38" priority="52">
+    <cfRule type="expression" dxfId="32" priority="53">
+      <formula>H3="In Process"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="31" priority="52">
       <formula>H3="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="53">
-      <formula>H3="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="36" priority="54">
+    <cfRule type="expression" dxfId="30" priority="54">
       <formula>H3="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
-    <cfRule type="expression" dxfId="35" priority="36">
-      <formula>H29="Not Started"</formula>
+  <conditionalFormatting sqref="M17">
+    <cfRule type="expression" dxfId="29" priority="33">
+      <formula>M17="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="35">
-      <formula>H29="In Process"</formula>
+    <cfRule type="expression" dxfId="28" priority="31">
+      <formula>M17="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="34">
-      <formula>H29="Completed"</formula>
+    <cfRule type="expression" dxfId="27" priority="30">
+      <formula>M17="Not Started"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M17">
-    <cfRule type="expression" dxfId="32" priority="32">
+    <cfRule type="expression" dxfId="26" priority="29">
       <formula>M17="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="31">
+    <cfRule type="expression" dxfId="25" priority="28">
       <formula>M17="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="30">
-      <formula>M17="Not Started"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="29" priority="29">
+    <cfRule type="expression" dxfId="24" priority="32">
       <formula>M17="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="28">
-      <formula>M17="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="33">
-      <formula>M17="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M19">
-    <cfRule type="expression" dxfId="26" priority="14">
+    <cfRule type="expression" dxfId="23" priority="10">
+      <formula>M19="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="11">
       <formula>M19="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="10">
-      <formula>M19="Completed"</formula>
+    <cfRule type="expression" dxfId="21" priority="12">
+      <formula>M19="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="11">
+    <cfRule type="expression" dxfId="20" priority="14">
       <formula>M19="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="12">
+    <cfRule type="expression" dxfId="19" priority="15">
       <formula>M19="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="13">
+    <cfRule type="expression" dxfId="18" priority="13">
       <formula>M19="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="21" priority="15">
-      <formula>M19="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M21">
-    <cfRule type="expression" dxfId="20" priority="4">
-      <formula>M21="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="5">
-      <formula>M21="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="6">
-      <formula>M21="Not Started"</formula>
-    </cfRule>
     <cfRule type="expression" dxfId="17" priority="7">
       <formula>M21="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="8">
+    <cfRule type="expression" dxfId="16" priority="9">
+      <formula>M21="Not Started"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="8">
       <formula>M21="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="9">
+    <cfRule type="expression" dxfId="14" priority="6">
       <formula>M21="Not Started"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="5">
+      <formula>M21="In Process"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="4">
+      <formula>M21="Completed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O17">
-    <cfRule type="expression" dxfId="14" priority="26">
+    <cfRule type="expression" dxfId="11" priority="27">
+      <formula>O17="Not Started"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="25">
+      <formula>O17="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="24">
+      <formula>O17="Not Started"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="23">
       <formula>O17="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="25">
+    <cfRule type="expression" dxfId="7" priority="22">
       <formula>O17="Completed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="24">
-      <formula>O17="Not Started"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="11" priority="23">
+    <cfRule type="expression" dxfId="6" priority="26">
       <formula>O17="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="27">
-      <formula>O17="Not Started"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="22">
-      <formula>O17="Completed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q17">
-    <cfRule type="expression" dxfId="8" priority="21">
+    <cfRule type="expression" dxfId="5" priority="20">
+      <formula>Q17="In Process"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="21">
       <formula>Q17="Not Started"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="20">
+    <cfRule type="expression" dxfId="3" priority="19">
+      <formula>Q17="Completed"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="18">
+      <formula>Q17="Not Started"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="17">
       <formula>Q17="In Process"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="19">
+    <cfRule type="expression" dxfId="0" priority="16">
       <formula>Q17="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="18">
-      <formula>Q17="Not Started"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="17">
-      <formula>Q17="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="16">
-      <formula>Q17="Completed"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>H30="Completed"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>H30="In Process"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
-      <formula>H30="Not Started"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -4440,14 +4354,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="8" customFormat="1" ht="0.2" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="113" t="s">
+      <c r="A1" s="126" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="113"/>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
     </row>
     <row r="2" spans="1:6" ht="0.2" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4"/>

</xml_diff>

<commit_message>
Updated documents in support of I-20 — Configuration Separation implementation.
</commit_message>
<xml_diff>
--- a/planing/implementation-plan/azure-policy-assist-prioritized-implementation-log-v12.xlsx
+++ b/planing/implementation-plan/azure-policy-assist-prioritized-implementation-log-v12.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steven\GitHub-Repositories\Repositories\azure-policy-assistant-rag-solution-docs\planing\implementation-plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F97FA7E2-C76F-468D-AC28-8B8E86D70550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51A8526-50DE-4070-BA2D-3115A2EADCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3724,19 +3724,19 @@
       <c r="E31" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F31" s="112" t="s">
+      <c r="F31" s="127" t="s">
         <v>168</v>
       </c>
-      <c r="G31" s="113" t="s">
+      <c r="G31" s="128" t="s">
         <v>169</v>
       </c>
       <c r="H31" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="I31" s="113" t="s">
+        <v>16</v>
+      </c>
+      <c r="I31" s="128" t="s">
         <v>170</v>
       </c>
-      <c r="J31" s="113" t="s">
+      <c r="J31" s="128" t="s">
         <v>171</v>
       </c>
     </row>
@@ -3756,19 +3756,19 @@
       <c r="E32" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="F32" s="56" t="s">
+      <c r="F32" s="112" t="s">
         <v>174</v>
       </c>
-      <c r="G32" s="57" t="s">
+      <c r="G32" s="113" t="s">
         <v>175</v>
       </c>
-      <c r="H32" s="55" t="s">
-        <v>118</v>
-      </c>
-      <c r="I32" s="57" t="s">
+      <c r="H32" s="49" t="s">
+        <v>107</v>
+      </c>
+      <c r="I32" s="113" t="s">
         <v>160</v>
       </c>
-      <c r="J32" s="57" t="s">
+      <c r="J32" s="113" t="s">
         <v>176</v>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       <formula>B3="P0"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H31">
+  <conditionalFormatting sqref="H3:H32">
     <cfRule type="expression" dxfId="35" priority="1">
       <formula>H3="Completed"</formula>
     </cfRule>

</xml_diff>